<commit_message>
docs: actualizar plantilla de importación
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plantilla_importacion.xlsx
+++ b/docs/plantilla_importacion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfranco\workspace-it\wordpress\buscador-parroquias\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF12736A-30C6-4C75-B032-F3BDC462A93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3DF545D-632A-4D80-AF48-68759EB63CCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F7231939-C397-4128-B389-6DABFCA65E7B}"/>
+    <workbookView xWindow="-28920" yWindow="-2940" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F7231939-C397-4128-B389-6DABFCA65E7B}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="2" r:id="rId1"/>
@@ -290,7 +290,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -298,6 +298,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -769,8 +770,8 @@
     <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="48.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.5703125" style="7" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
@@ -830,10 +831,10 @@
       <c r="D2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>17</v>
       </c>
       <c r="G2" s="4" t="s">
@@ -868,10 +869,10 @@
       <c r="D3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>27</v>
       </c>
       <c r="G3" s="6" t="s">
@@ -906,10 +907,10 @@
       <c r="D4" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>36</v>
       </c>
       <c r="G4" s="4" t="s">

</xml_diff>